<commit_message>
Clarify international WhatsApp format in guest entry and Excel
</commit_message>
<xml_diff>
--- a/public/templates/plantilla-invitados.xlsx
+++ b/public/templates/plantilla-invitados.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Invitados" sheetId="1" r:id="Rabf4c259a35d4a71"/>
+    <sheet name="Invitados" sheetId="1" r:id="Rf4d67ed31f6249d8"/>
   </sheets>
 </workbook>
 </file>
@@ -435,7 +435,7 @@
     </row>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="5" t="str">
-        <v>Completa tu lista, guarda el archivo y súbelo a tu evento.</v>
+        <v>WhatsApp: incluye + y el código de país, sin espacios. Perú: +51987654321. Usa el código de cada país.</v>
       </c>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>

</xml_diff>

<commit_message>
Limit country pickers to Spanish-speaking markets and the United States
</commit_message>
<xml_diff>
--- a/public/templates/plantilla-invitados.xlsx
+++ b/public/templates/plantilla-invitados.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Invitados" sheetId="1" r:id="R6b73a0ac8cb44eb7"/>
-    <sheet name="Países" sheetId="2" r:id="R0d6539ea5a2546f1" state="hidden"/>
+    <sheet name="Invitados" sheetId="1" r:id="R8ec6eedff6db497f"/>
+    <sheet name="Países" sheetId="2" r:id="Rc3469867abcc486d" state="hidden"/>
   </sheets>
   <definedNames>
-    <definedName name="PaisesTelefonicos">'Países'!$A$2:$A$246</definedName>
+    <definedName name="PaisesTelefonicos">'Países'!$A$2:$A$22</definedName>
   </definedNames>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -530,7 +530,7 @@
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
       <c r="G5" s="9" t="str">
-        <f>IFERROR(IF($D$5="","",_xlfn.IMAGE("https://flagcdn.com/w80/"&amp;LOWER(VLOOKUP($D$5,'Países'!$A$2:$C$246,2,FALSE))&amp;".png","Bandera del país",0)),"")</f>
+        <f>IFERROR(IF($D$5="","",_xlfn.IMAGE("https://flagcdn.com/w80/"&amp;LOWER(VLOOKUP($D$5,'Países'!$A$2:$C$22,2,FALSE))&amp;".png","Bandera del país",0)),"")</f>
       </c>
       <c r="H5" s="6"/>
     </row>
@@ -6659,197 +6659,197 @@
     </row>
     <row r="2" ht="23" customHeight="1">
       <c r="A2" s="1" t="str">
-        <v>Afganistán (+93)</v>
+        <v>Argentina (+54)</v>
       </c>
       <c r="B2" s="1" t="str">
-        <v>AF</v>
+        <v>AR</v>
       </c>
       <c r="C2" s="1" t="str">
-        <v>+93</v>
+        <v>+54</v>
       </c>
     </row>
     <row r="3" ht="23" customHeight="1">
       <c r="A3" s="1" t="str">
-        <v>Albania (+355)</v>
+        <v>Bolivia (+591)</v>
       </c>
       <c r="B3" s="1" t="str">
-        <v>AL</v>
+        <v>BO</v>
       </c>
       <c r="C3" s="1" t="str">
-        <v>+355</v>
+        <v>+591</v>
       </c>
     </row>
     <row r="4" ht="23" customHeight="1">
       <c r="A4" s="1" t="str">
-        <v>Alemania (+49)</v>
+        <v>Chile (+56)</v>
       </c>
       <c r="B4" s="1" t="str">
-        <v>DE</v>
+        <v>CL</v>
       </c>
       <c r="C4" s="1" t="str">
-        <v>+49</v>
+        <v>+56</v>
       </c>
     </row>
     <row r="5" ht="23" customHeight="1">
       <c r="A5" s="1" t="str">
-        <v>Andorra (+376)</v>
+        <v>Colombia (+57)</v>
       </c>
       <c r="B5" s="1" t="str">
-        <v>AD</v>
+        <v>CO</v>
       </c>
       <c r="C5" s="1" t="str">
-        <v>+376</v>
+        <v>+57</v>
       </c>
     </row>
     <row r="6" ht="23" customHeight="1">
       <c r="A6" s="1" t="str">
-        <v>Angola (+244)</v>
+        <v>Costa Rica (+506)</v>
       </c>
       <c r="B6" s="1" t="str">
-        <v>AO</v>
+        <v>CR</v>
       </c>
       <c r="C6" s="1" t="str">
-        <v>+244</v>
+        <v>+506</v>
       </c>
     </row>
     <row r="7" ht="23" customHeight="1">
       <c r="A7" s="1" t="str">
-        <v>Anguila (+1)</v>
+        <v>Cuba (+53)</v>
       </c>
       <c r="B7" s="1" t="str">
-        <v>AI</v>
+        <v>CU</v>
       </c>
       <c r="C7" s="1" t="str">
-        <v>+1</v>
+        <v>+53</v>
       </c>
     </row>
     <row r="8" ht="23" customHeight="1">
       <c r="A8" s="1" t="str">
-        <v>Antigua y Barbuda (+1)</v>
+        <v>Ecuador (+593)</v>
       </c>
       <c r="B8" s="1" t="str">
-        <v>AG</v>
+        <v>EC</v>
       </c>
       <c r="C8" s="1" t="str">
-        <v>+1</v>
+        <v>+593</v>
       </c>
     </row>
     <row r="9" ht="23" customHeight="1">
       <c r="A9" s="1" t="str">
-        <v>Arabia Saudí (+966)</v>
+        <v>El Salvador (+503)</v>
       </c>
       <c r="B9" s="1" t="str">
-        <v>SA</v>
+        <v>SV</v>
       </c>
       <c r="C9" s="1" t="str">
-        <v>+966</v>
+        <v>+503</v>
       </c>
     </row>
     <row r="10" ht="23" customHeight="1">
       <c r="A10" s="1" t="str">
-        <v>Argelia (+213)</v>
+        <v>España (+34)</v>
       </c>
       <c r="B10" s="1" t="str">
-        <v>DZ</v>
+        <v>ES</v>
       </c>
       <c r="C10" s="1" t="str">
-        <v>+213</v>
+        <v>+34</v>
       </c>
     </row>
     <row r="11" ht="23" customHeight="1">
       <c r="A11" s="1" t="str">
-        <v>Argentina (+54)</v>
+        <v>Estados Unidos (+1)</v>
       </c>
       <c r="B11" s="1" t="str">
-        <v>AR</v>
+        <v>US</v>
       </c>
       <c r="C11" s="1" t="str">
-        <v>+54</v>
+        <v>+1</v>
       </c>
     </row>
     <row r="12" ht="23" customHeight="1">
       <c r="A12" s="1" t="str">
-        <v>Armenia (+374)</v>
+        <v>Guatemala (+502)</v>
       </c>
       <c r="B12" s="1" t="str">
-        <v>AM</v>
+        <v>GT</v>
       </c>
       <c r="C12" s="1" t="str">
-        <v>+374</v>
+        <v>+502</v>
       </c>
     </row>
     <row r="13" ht="23" customHeight="1">
       <c r="A13" s="1" t="str">
-        <v>Aruba (+297)</v>
+        <v>Honduras (+504)</v>
       </c>
       <c r="B13" s="1" t="str">
-        <v>AW</v>
+        <v>HN</v>
       </c>
       <c r="C13" s="1" t="str">
-        <v>+297</v>
+        <v>+504</v>
       </c>
     </row>
     <row r="14" ht="23" customHeight="1">
       <c r="A14" s="1" t="str">
-        <v>Australia (+61)</v>
+        <v>México (+52)</v>
       </c>
       <c r="B14" s="1" t="str">
-        <v>AU</v>
+        <v>MX</v>
       </c>
       <c r="C14" s="1" t="str">
-        <v>+61</v>
+        <v>+52</v>
       </c>
     </row>
     <row r="15" ht="23" customHeight="1">
       <c r="A15" s="1" t="str">
-        <v>Austria (+43)</v>
+        <v>Nicaragua (+505)</v>
       </c>
       <c r="B15" s="1" t="str">
-        <v>AT</v>
+        <v>NI</v>
       </c>
       <c r="C15" s="1" t="str">
-        <v>+43</v>
+        <v>+505</v>
       </c>
     </row>
     <row r="16" ht="23" customHeight="1">
       <c r="A16" s="1" t="str">
-        <v>Azerbaiyán (+994)</v>
+        <v>Panamá (+507)</v>
       </c>
       <c r="B16" s="1" t="str">
-        <v>AZ</v>
+        <v>PA</v>
       </c>
       <c r="C16" s="1" t="str">
-        <v>+994</v>
+        <v>+507</v>
       </c>
     </row>
     <row r="17" ht="23" customHeight="1">
       <c r="A17" s="1" t="str">
-        <v>Bahamas (+1)</v>
+        <v>Paraguay (+595)</v>
       </c>
       <c r="B17" s="1" t="str">
-        <v>BS</v>
+        <v>PY</v>
       </c>
       <c r="C17" s="1" t="str">
-        <v>+1</v>
+        <v>+595</v>
       </c>
     </row>
     <row r="18" ht="23" customHeight="1">
       <c r="A18" s="1" t="str">
-        <v>Bangladés (+880)</v>
+        <v>Perú (+51)</v>
       </c>
       <c r="B18" s="1" t="str">
-        <v>BD</v>
+        <v>PE</v>
       </c>
       <c r="C18" s="1" t="str">
-        <v>+880</v>
+        <v>+51</v>
       </c>
     </row>
     <row r="19" ht="23" customHeight="1">
       <c r="A19" s="1" t="str">
-        <v>Barbados (+1)</v>
+        <v>Puerto Rico (+1)</v>
       </c>
       <c r="B19" s="1" t="str">
-        <v>BB</v>
+        <v>PR</v>
       </c>
       <c r="C19" s="1" t="str">
         <v>+1</v>
@@ -6857,2499 +6857,35 @@
     </row>
     <row r="20" ht="23" customHeight="1">
       <c r="A20" s="1" t="str">
-        <v>Baréin (+973)</v>
+        <v>República Dominicana (+1)</v>
       </c>
       <c r="B20" s="1" t="str">
-        <v>BH</v>
+        <v>DO</v>
       </c>
       <c r="C20" s="1" t="str">
-        <v>+973</v>
+        <v>+1</v>
       </c>
     </row>
     <row r="21" ht="23" customHeight="1">
       <c r="A21" s="1" t="str">
-        <v>Bélgica (+32)</v>
+        <v>Uruguay (+598)</v>
       </c>
       <c r="B21" s="1" t="str">
-        <v>BE</v>
+        <v>UY</v>
       </c>
       <c r="C21" s="1" t="str">
-        <v>+32</v>
+        <v>+598</v>
       </c>
     </row>
     <row r="22" ht="23" customHeight="1">
       <c r="A22" s="1" t="str">
-        <v>Belice (+501)</v>
+        <v>Venezuela (+58)</v>
       </c>
       <c r="B22" s="1" t="str">
-        <v>BZ</v>
+        <v>VE</v>
       </c>
       <c r="C22" s="1" t="str">
-        <v>+501</v>
-      </c>
-    </row>
-    <row r="23" ht="23" customHeight="1">
-      <c r="A23" s="1" t="str">
-        <v>Benín (+229)</v>
-      </c>
-      <c r="B23" s="1" t="str">
-        <v>BJ</v>
-      </c>
-      <c r="C23" s="1" t="str">
-        <v>+229</v>
-      </c>
-    </row>
-    <row r="24" ht="23" customHeight="1">
-      <c r="A24" s="1" t="str">
-        <v>Bermudas (+1)</v>
-      </c>
-      <c r="B24" s="1" t="str">
-        <v>BM</v>
-      </c>
-      <c r="C24" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="25" ht="23" customHeight="1">
-      <c r="A25" s="1" t="str">
-        <v>Bielorrusia (+375)</v>
-      </c>
-      <c r="B25" s="1" t="str">
-        <v>BY</v>
-      </c>
-      <c r="C25" s="1" t="str">
-        <v>+375</v>
-      </c>
-    </row>
-    <row r="26" ht="23" customHeight="1">
-      <c r="A26" s="1" t="str">
-        <v>Bolivia (+591)</v>
-      </c>
-      <c r="B26" s="1" t="str">
-        <v>BO</v>
-      </c>
-      <c r="C26" s="1" t="str">
-        <v>+591</v>
-      </c>
-    </row>
-    <row r="27" ht="23" customHeight="1">
-      <c r="A27" s="1" t="str">
-        <v>Bosnia y Herzegovina (+387)</v>
-      </c>
-      <c r="B27" s="1" t="str">
-        <v>BA</v>
-      </c>
-      <c r="C27" s="1" t="str">
-        <v>+387</v>
-      </c>
-    </row>
-    <row r="28" ht="23" customHeight="1">
-      <c r="A28" s="1" t="str">
-        <v>Botsuana (+267)</v>
-      </c>
-      <c r="B28" s="1" t="str">
-        <v>BW</v>
-      </c>
-      <c r="C28" s="1" t="str">
-        <v>+267</v>
-      </c>
-    </row>
-    <row r="29" ht="23" customHeight="1">
-      <c r="A29" s="1" t="str">
-        <v>Brasil (+55)</v>
-      </c>
-      <c r="B29" s="1" t="str">
-        <v>BR</v>
-      </c>
-      <c r="C29" s="1" t="str">
-        <v>+55</v>
-      </c>
-    </row>
-    <row r="30" ht="23" customHeight="1">
-      <c r="A30" s="1" t="str">
-        <v>Brunéi (+673)</v>
-      </c>
-      <c r="B30" s="1" t="str">
-        <v>BN</v>
-      </c>
-      <c r="C30" s="1" t="str">
-        <v>+673</v>
-      </c>
-    </row>
-    <row r="31" ht="23" customHeight="1">
-      <c r="A31" s="1" t="str">
-        <v>Bulgaria (+359)</v>
-      </c>
-      <c r="B31" s="1" t="str">
-        <v>BG</v>
-      </c>
-      <c r="C31" s="1" t="str">
-        <v>+359</v>
-      </c>
-    </row>
-    <row r="32" ht="23" customHeight="1">
-      <c r="A32" s="1" t="str">
-        <v>Burkina Faso (+226)</v>
-      </c>
-      <c r="B32" s="1" t="str">
-        <v>BF</v>
-      </c>
-      <c r="C32" s="1" t="str">
-        <v>+226</v>
-      </c>
-    </row>
-    <row r="33" ht="23" customHeight="1">
-      <c r="A33" s="1" t="str">
-        <v>Burundi (+257)</v>
-      </c>
-      <c r="B33" s="1" t="str">
-        <v>BI</v>
-      </c>
-      <c r="C33" s="1" t="str">
-        <v>+257</v>
-      </c>
-    </row>
-    <row r="34" ht="23" customHeight="1">
-      <c r="A34" s="1" t="str">
-        <v>Bután (+975)</v>
-      </c>
-      <c r="B34" s="1" t="str">
-        <v>BT</v>
-      </c>
-      <c r="C34" s="1" t="str">
-        <v>+975</v>
-      </c>
-    </row>
-    <row r="35" ht="23" customHeight="1">
-      <c r="A35" s="1" t="str">
-        <v>Cabo Verde (+238)</v>
-      </c>
-      <c r="B35" s="1" t="str">
-        <v>CV</v>
-      </c>
-      <c r="C35" s="1" t="str">
-        <v>+238</v>
-      </c>
-    </row>
-    <row r="36" ht="23" customHeight="1">
-      <c r="A36" s="1" t="str">
-        <v>Camboya (+855)</v>
-      </c>
-      <c r="B36" s="1" t="str">
-        <v>KH</v>
-      </c>
-      <c r="C36" s="1" t="str">
-        <v>+855</v>
-      </c>
-    </row>
-    <row r="37" ht="23" customHeight="1">
-      <c r="A37" s="1" t="str">
-        <v>Camerún (+237)</v>
-      </c>
-      <c r="B37" s="1" t="str">
-        <v>CM</v>
-      </c>
-      <c r="C37" s="1" t="str">
-        <v>+237</v>
-      </c>
-    </row>
-    <row r="38" ht="23" customHeight="1">
-      <c r="A38" s="1" t="str">
-        <v>Canadá (+1)</v>
-      </c>
-      <c r="B38" s="1" t="str">
-        <v>CA</v>
-      </c>
-      <c r="C38" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="39" ht="23" customHeight="1">
-      <c r="A39" s="1" t="str">
-        <v>Caribe neerlandés (+599)</v>
-      </c>
-      <c r="B39" s="1" t="str">
-        <v>BQ</v>
-      </c>
-      <c r="C39" s="1" t="str">
-        <v>+599</v>
-      </c>
-    </row>
-    <row r="40" ht="23" customHeight="1">
-      <c r="A40" s="1" t="str">
-        <v>Catar (+974)</v>
-      </c>
-      <c r="B40" s="1" t="str">
-        <v>QA</v>
-      </c>
-      <c r="C40" s="1" t="str">
-        <v>+974</v>
-      </c>
-    </row>
-    <row r="41" ht="23" customHeight="1">
-      <c r="A41" s="1" t="str">
-        <v>Chad (+235)</v>
-      </c>
-      <c r="B41" s="1" t="str">
-        <v>TD</v>
-      </c>
-      <c r="C41" s="1" t="str">
-        <v>+235</v>
-      </c>
-    </row>
-    <row r="42" ht="23" customHeight="1">
-      <c r="A42" s="1" t="str">
-        <v>Chequia (+420)</v>
-      </c>
-      <c r="B42" s="1" t="str">
-        <v>CZ</v>
-      </c>
-      <c r="C42" s="1" t="str">
-        <v>+420</v>
-      </c>
-    </row>
-    <row r="43" ht="23" customHeight="1">
-      <c r="A43" s="1" t="str">
-        <v>Chile (+56)</v>
-      </c>
-      <c r="B43" s="1" t="str">
-        <v>CL</v>
-      </c>
-      <c r="C43" s="1" t="str">
-        <v>+56</v>
-      </c>
-    </row>
-    <row r="44" ht="23" customHeight="1">
-      <c r="A44" s="1" t="str">
-        <v>China (+86)</v>
-      </c>
-      <c r="B44" s="1" t="str">
-        <v>CN</v>
-      </c>
-      <c r="C44" s="1" t="str">
-        <v>+86</v>
-      </c>
-    </row>
-    <row r="45" ht="23" customHeight="1">
-      <c r="A45" s="1" t="str">
-        <v>Chipre (+357)</v>
-      </c>
-      <c r="B45" s="1" t="str">
-        <v>CY</v>
-      </c>
-      <c r="C45" s="1" t="str">
-        <v>+357</v>
-      </c>
-    </row>
-    <row r="46" ht="23" customHeight="1">
-      <c r="A46" s="1" t="str">
-        <v>Ciudad del Vaticano (+39)</v>
-      </c>
-      <c r="B46" s="1" t="str">
-        <v>VA</v>
-      </c>
-      <c r="C46" s="1" t="str">
-        <v>+39</v>
-      </c>
-    </row>
-    <row r="47" ht="23" customHeight="1">
-      <c r="A47" s="1" t="str">
-        <v>Colombia (+57)</v>
-      </c>
-      <c r="B47" s="1" t="str">
-        <v>CO</v>
-      </c>
-      <c r="C47" s="1" t="str">
-        <v>+57</v>
-      </c>
-    </row>
-    <row r="48" ht="23" customHeight="1">
-      <c r="A48" s="1" t="str">
-        <v>Comoras (+269)</v>
-      </c>
-      <c r="B48" s="1" t="str">
-        <v>KM</v>
-      </c>
-      <c r="C48" s="1" t="str">
-        <v>+269</v>
-      </c>
-    </row>
-    <row r="49" ht="23" customHeight="1">
-      <c r="A49" s="1" t="str">
-        <v>Congo (+242)</v>
-      </c>
-      <c r="B49" s="1" t="str">
-        <v>CG</v>
-      </c>
-      <c r="C49" s="1" t="str">
-        <v>+242</v>
-      </c>
-    </row>
-    <row r="50" ht="23" customHeight="1">
-      <c r="A50" s="1" t="str">
-        <v>Corea del Norte (+850)</v>
-      </c>
-      <c r="B50" s="1" t="str">
-        <v>KP</v>
-      </c>
-      <c r="C50" s="1" t="str">
-        <v>+850</v>
-      </c>
-    </row>
-    <row r="51" ht="23" customHeight="1">
-      <c r="A51" s="1" t="str">
-        <v>Corea del Sur (+82)</v>
-      </c>
-      <c r="B51" s="1" t="str">
-        <v>KR</v>
-      </c>
-      <c r="C51" s="1" t="str">
-        <v>+82</v>
-      </c>
-    </row>
-    <row r="52" ht="23" customHeight="1">
-      <c r="A52" s="1" t="str">
-        <v>Costa Rica (+506)</v>
-      </c>
-      <c r="B52" s="1" t="str">
-        <v>CR</v>
-      </c>
-      <c r="C52" s="1" t="str">
-        <v>+506</v>
-      </c>
-    </row>
-    <row r="53" ht="23" customHeight="1">
-      <c r="A53" s="1" t="str">
-        <v>Côte d’Ivoire (+225)</v>
-      </c>
-      <c r="B53" s="1" t="str">
-        <v>CI</v>
-      </c>
-      <c r="C53" s="1" t="str">
-        <v>+225</v>
-      </c>
-    </row>
-    <row r="54" ht="23" customHeight="1">
-      <c r="A54" s="1" t="str">
-        <v>Croacia (+385)</v>
-      </c>
-      <c r="B54" s="1" t="str">
-        <v>HR</v>
-      </c>
-      <c r="C54" s="1" t="str">
-        <v>+385</v>
-      </c>
-    </row>
-    <row r="55" ht="23" customHeight="1">
-      <c r="A55" s="1" t="str">
-        <v>Cuba (+53)</v>
-      </c>
-      <c r="B55" s="1" t="str">
-        <v>CU</v>
-      </c>
-      <c r="C55" s="1" t="str">
-        <v>+53</v>
-      </c>
-    </row>
-    <row r="56" ht="23" customHeight="1">
-      <c r="A56" s="1" t="str">
-        <v>Curazao (+599)</v>
-      </c>
-      <c r="B56" s="1" t="str">
-        <v>CW</v>
-      </c>
-      <c r="C56" s="1" t="str">
-        <v>+599</v>
-      </c>
-    </row>
-    <row r="57" ht="23" customHeight="1">
-      <c r="A57" s="1" t="str">
-        <v>Dinamarca (+45)</v>
-      </c>
-      <c r="B57" s="1" t="str">
-        <v>DK</v>
-      </c>
-      <c r="C57" s="1" t="str">
-        <v>+45</v>
-      </c>
-    </row>
-    <row r="58" ht="23" customHeight="1">
-      <c r="A58" s="1" t="str">
-        <v>Dominica (+1)</v>
-      </c>
-      <c r="B58" s="1" t="str">
-        <v>DM</v>
-      </c>
-      <c r="C58" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="59" ht="23" customHeight="1">
-      <c r="A59" s="1" t="str">
-        <v>Ecuador (+593)</v>
-      </c>
-      <c r="B59" s="1" t="str">
-        <v>EC</v>
-      </c>
-      <c r="C59" s="1" t="str">
-        <v>+593</v>
-      </c>
-    </row>
-    <row r="60" ht="23" customHeight="1">
-      <c r="A60" s="1" t="str">
-        <v>Egipto (+20)</v>
-      </c>
-      <c r="B60" s="1" t="str">
-        <v>EG</v>
-      </c>
-      <c r="C60" s="1" t="str">
-        <v>+20</v>
-      </c>
-    </row>
-    <row r="61" ht="23" customHeight="1">
-      <c r="A61" s="1" t="str">
-        <v>El Salvador (+503)</v>
-      </c>
-      <c r="B61" s="1" t="str">
-        <v>SV</v>
-      </c>
-      <c r="C61" s="1" t="str">
-        <v>+503</v>
-      </c>
-    </row>
-    <row r="62" ht="23" customHeight="1">
-      <c r="A62" s="1" t="str">
-        <v>Emiratos Árabes Unidos (+971)</v>
-      </c>
-      <c r="B62" s="1" t="str">
-        <v>AE</v>
-      </c>
-      <c r="C62" s="1" t="str">
-        <v>+971</v>
-      </c>
-    </row>
-    <row r="63" ht="23" customHeight="1">
-      <c r="A63" s="1" t="str">
-        <v>Eritrea (+291)</v>
-      </c>
-      <c r="B63" s="1" t="str">
-        <v>ER</v>
-      </c>
-      <c r="C63" s="1" t="str">
-        <v>+291</v>
-      </c>
-    </row>
-    <row r="64" ht="23" customHeight="1">
-      <c r="A64" s="1" t="str">
-        <v>Eslovaquia (+421)</v>
-      </c>
-      <c r="B64" s="1" t="str">
-        <v>SK</v>
-      </c>
-      <c r="C64" s="1" t="str">
-        <v>+421</v>
-      </c>
-    </row>
-    <row r="65" ht="23" customHeight="1">
-      <c r="A65" s="1" t="str">
-        <v>Eslovenia (+386)</v>
-      </c>
-      <c r="B65" s="1" t="str">
-        <v>SI</v>
-      </c>
-      <c r="C65" s="1" t="str">
-        <v>+386</v>
-      </c>
-    </row>
-    <row r="66" ht="23" customHeight="1">
-      <c r="A66" s="1" t="str">
-        <v>España (+34)</v>
-      </c>
-      <c r="B66" s="1" t="str">
-        <v>ES</v>
-      </c>
-      <c r="C66" s="1" t="str">
-        <v>+34</v>
-      </c>
-    </row>
-    <row r="67" ht="23" customHeight="1">
-      <c r="A67" s="1" t="str">
-        <v>Estados Unidos (+1)</v>
-      </c>
-      <c r="B67" s="1" t="str">
-        <v>US</v>
-      </c>
-      <c r="C67" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="68" ht="23" customHeight="1">
-      <c r="A68" s="1" t="str">
-        <v>Estonia (+372)</v>
-      </c>
-      <c r="B68" s="1" t="str">
-        <v>EE</v>
-      </c>
-      <c r="C68" s="1" t="str">
-        <v>+372</v>
-      </c>
-    </row>
-    <row r="69" ht="23" customHeight="1">
-      <c r="A69" s="1" t="str">
-        <v>Esuatini (+268)</v>
-      </c>
-      <c r="B69" s="1" t="str">
-        <v>SZ</v>
-      </c>
-      <c r="C69" s="1" t="str">
-        <v>+268</v>
-      </c>
-    </row>
-    <row r="70" ht="23" customHeight="1">
-      <c r="A70" s="1" t="str">
-        <v>Etiopía (+251)</v>
-      </c>
-      <c r="B70" s="1" t="str">
-        <v>ET</v>
-      </c>
-      <c r="C70" s="1" t="str">
-        <v>+251</v>
-      </c>
-    </row>
-    <row r="71" ht="23" customHeight="1">
-      <c r="A71" s="1" t="str">
-        <v>Filipinas (+63)</v>
-      </c>
-      <c r="B71" s="1" t="str">
-        <v>PH</v>
-      </c>
-      <c r="C71" s="1" t="str">
-        <v>+63</v>
-      </c>
-    </row>
-    <row r="72" ht="23" customHeight="1">
-      <c r="A72" s="1" t="str">
-        <v>Finlandia (+358)</v>
-      </c>
-      <c r="B72" s="1" t="str">
-        <v>FI</v>
-      </c>
-      <c r="C72" s="1" t="str">
-        <v>+358</v>
-      </c>
-    </row>
-    <row r="73" ht="23" customHeight="1">
-      <c r="A73" s="1" t="str">
-        <v>Fiyi (+679)</v>
-      </c>
-      <c r="B73" s="1" t="str">
-        <v>FJ</v>
-      </c>
-      <c r="C73" s="1" t="str">
-        <v>+679</v>
-      </c>
-    </row>
-    <row r="74" ht="23" customHeight="1">
-      <c r="A74" s="1" t="str">
-        <v>Francia (+33)</v>
-      </c>
-      <c r="B74" s="1" t="str">
-        <v>FR</v>
-      </c>
-      <c r="C74" s="1" t="str">
-        <v>+33</v>
-      </c>
-    </row>
-    <row r="75" ht="23" customHeight="1">
-      <c r="A75" s="1" t="str">
-        <v>Gabón (+241)</v>
-      </c>
-      <c r="B75" s="1" t="str">
-        <v>GA</v>
-      </c>
-      <c r="C75" s="1" t="str">
-        <v>+241</v>
-      </c>
-    </row>
-    <row r="76" ht="23" customHeight="1">
-      <c r="A76" s="1" t="str">
-        <v>Gambia (+220)</v>
-      </c>
-      <c r="B76" s="1" t="str">
-        <v>GM</v>
-      </c>
-      <c r="C76" s="1" t="str">
-        <v>+220</v>
-      </c>
-    </row>
-    <row r="77" ht="23" customHeight="1">
-      <c r="A77" s="1" t="str">
-        <v>Georgia (+995)</v>
-      </c>
-      <c r="B77" s="1" t="str">
-        <v>GE</v>
-      </c>
-      <c r="C77" s="1" t="str">
-        <v>+995</v>
-      </c>
-    </row>
-    <row r="78" ht="23" customHeight="1">
-      <c r="A78" s="1" t="str">
-        <v>Ghana (+233)</v>
-      </c>
-      <c r="B78" s="1" t="str">
-        <v>GH</v>
-      </c>
-      <c r="C78" s="1" t="str">
-        <v>+233</v>
-      </c>
-    </row>
-    <row r="79" ht="23" customHeight="1">
-      <c r="A79" s="1" t="str">
-        <v>Gibraltar (+350)</v>
-      </c>
-      <c r="B79" s="1" t="str">
-        <v>GI</v>
-      </c>
-      <c r="C79" s="1" t="str">
-        <v>+350</v>
-      </c>
-    </row>
-    <row r="80" ht="23" customHeight="1">
-      <c r="A80" s="1" t="str">
-        <v>Granada (+1)</v>
-      </c>
-      <c r="B80" s="1" t="str">
-        <v>GD</v>
-      </c>
-      <c r="C80" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="81" ht="23" customHeight="1">
-      <c r="A81" s="1" t="str">
-        <v>Grecia (+30)</v>
-      </c>
-      <c r="B81" s="1" t="str">
-        <v>GR</v>
-      </c>
-      <c r="C81" s="1" t="str">
-        <v>+30</v>
-      </c>
-    </row>
-    <row r="82" ht="23" customHeight="1">
-      <c r="A82" s="1" t="str">
-        <v>Groenlandia (+299)</v>
-      </c>
-      <c r="B82" s="1" t="str">
-        <v>GL</v>
-      </c>
-      <c r="C82" s="1" t="str">
-        <v>+299</v>
-      </c>
-    </row>
-    <row r="83" ht="23" customHeight="1">
-      <c r="A83" s="1" t="str">
-        <v>Guadalupe (+590)</v>
-      </c>
-      <c r="B83" s="1" t="str">
-        <v>GP</v>
-      </c>
-      <c r="C83" s="1" t="str">
-        <v>+590</v>
-      </c>
-    </row>
-    <row r="84" ht="23" customHeight="1">
-      <c r="A84" s="1" t="str">
-        <v>Guam (+1)</v>
-      </c>
-      <c r="B84" s="1" t="str">
-        <v>GU</v>
-      </c>
-      <c r="C84" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="85" ht="23" customHeight="1">
-      <c r="A85" s="1" t="str">
-        <v>Guatemala (+502)</v>
-      </c>
-      <c r="B85" s="1" t="str">
-        <v>GT</v>
-      </c>
-      <c r="C85" s="1" t="str">
-        <v>+502</v>
-      </c>
-    </row>
-    <row r="86" ht="23" customHeight="1">
-      <c r="A86" s="1" t="str">
-        <v>Guayana Francesa (+594)</v>
-      </c>
-      <c r="B86" s="1" t="str">
-        <v>GF</v>
-      </c>
-      <c r="C86" s="1" t="str">
-        <v>+594</v>
-      </c>
-    </row>
-    <row r="87" ht="23" customHeight="1">
-      <c r="A87" s="1" t="str">
-        <v>Guernesey (+44)</v>
-      </c>
-      <c r="B87" s="1" t="str">
-        <v>GG</v>
-      </c>
-      <c r="C87" s="1" t="str">
-        <v>+44</v>
-      </c>
-    </row>
-    <row r="88" ht="23" customHeight="1">
-      <c r="A88" s="1" t="str">
-        <v>Guinea (+224)</v>
-      </c>
-      <c r="B88" s="1" t="str">
-        <v>GN</v>
-      </c>
-      <c r="C88" s="1" t="str">
-        <v>+224</v>
-      </c>
-    </row>
-    <row r="89" ht="23" customHeight="1">
-      <c r="A89" s="1" t="str">
-        <v>Guinea Ecuatorial (+240)</v>
-      </c>
-      <c r="B89" s="1" t="str">
-        <v>GQ</v>
-      </c>
-      <c r="C89" s="1" t="str">
-        <v>+240</v>
-      </c>
-    </row>
-    <row r="90" ht="23" customHeight="1">
-      <c r="A90" s="1" t="str">
-        <v>Guinea-Bisáu (+245)</v>
-      </c>
-      <c r="B90" s="1" t="str">
-        <v>GW</v>
-      </c>
-      <c r="C90" s="1" t="str">
-        <v>+245</v>
-      </c>
-    </row>
-    <row r="91" ht="23" customHeight="1">
-      <c r="A91" s="1" t="str">
-        <v>Guyana (+592)</v>
-      </c>
-      <c r="B91" s="1" t="str">
-        <v>GY</v>
-      </c>
-      <c r="C91" s="1" t="str">
-        <v>+592</v>
-      </c>
-    </row>
-    <row r="92" ht="23" customHeight="1">
-      <c r="A92" s="1" t="str">
-        <v>Haití (+509)</v>
-      </c>
-      <c r="B92" s="1" t="str">
-        <v>HT</v>
-      </c>
-      <c r="C92" s="1" t="str">
-        <v>+509</v>
-      </c>
-    </row>
-    <row r="93" ht="23" customHeight="1">
-      <c r="A93" s="1" t="str">
-        <v>Honduras (+504)</v>
-      </c>
-      <c r="B93" s="1" t="str">
-        <v>HN</v>
-      </c>
-      <c r="C93" s="1" t="str">
-        <v>+504</v>
-      </c>
-    </row>
-    <row r="94" ht="23" customHeight="1">
-      <c r="A94" s="1" t="str">
-        <v>Hungría (+36)</v>
-      </c>
-      <c r="B94" s="1" t="str">
-        <v>HU</v>
-      </c>
-      <c r="C94" s="1" t="str">
-        <v>+36</v>
-      </c>
-    </row>
-    <row r="95" ht="23" customHeight="1">
-      <c r="A95" s="1" t="str">
-        <v>India (+91)</v>
-      </c>
-      <c r="B95" s="1" t="str">
-        <v>IN</v>
-      </c>
-      <c r="C95" s="1" t="str">
-        <v>+91</v>
-      </c>
-    </row>
-    <row r="96" ht="23" customHeight="1">
-      <c r="A96" s="1" t="str">
-        <v>Indonesia (+62)</v>
-      </c>
-      <c r="B96" s="1" t="str">
-        <v>ID</v>
-      </c>
-      <c r="C96" s="1" t="str">
-        <v>+62</v>
-      </c>
-    </row>
-    <row r="97" ht="23" customHeight="1">
-      <c r="A97" s="1" t="str">
-        <v>Irak (+964)</v>
-      </c>
-      <c r="B97" s="1" t="str">
-        <v>IQ</v>
-      </c>
-      <c r="C97" s="1" t="str">
-        <v>+964</v>
-      </c>
-    </row>
-    <row r="98" ht="23" customHeight="1">
-      <c r="A98" s="1" t="str">
-        <v>Irán (+98)</v>
-      </c>
-      <c r="B98" s="1" t="str">
-        <v>IR</v>
-      </c>
-      <c r="C98" s="1" t="str">
-        <v>+98</v>
-      </c>
-    </row>
-    <row r="99" ht="23" customHeight="1">
-      <c r="A99" s="1" t="str">
-        <v>Irlanda (+353)</v>
-      </c>
-      <c r="B99" s="1" t="str">
-        <v>IE</v>
-      </c>
-      <c r="C99" s="1" t="str">
-        <v>+353</v>
-      </c>
-    </row>
-    <row r="100" ht="23" customHeight="1">
-      <c r="A100" s="1" t="str">
-        <v>Isla de la Ascensión (+247)</v>
-      </c>
-      <c r="B100" s="1" t="str">
-        <v>AC</v>
-      </c>
-      <c r="C100" s="1" t="str">
-        <v>+247</v>
-      </c>
-    </row>
-    <row r="101" ht="23" customHeight="1">
-      <c r="A101" s="1" t="str">
-        <v>Isla de Man (+44)</v>
-      </c>
-      <c r="B101" s="1" t="str">
-        <v>IM</v>
-      </c>
-      <c r="C101" s="1" t="str">
-        <v>+44</v>
-      </c>
-    </row>
-    <row r="102" ht="23" customHeight="1">
-      <c r="A102" s="1" t="str">
-        <v>Isla de Navidad (+61)</v>
-      </c>
-      <c r="B102" s="1" t="str">
-        <v>CX</v>
-      </c>
-      <c r="C102" s="1" t="str">
-        <v>+61</v>
-      </c>
-    </row>
-    <row r="103" ht="23" customHeight="1">
-      <c r="A103" s="1" t="str">
-        <v>Isla Norfolk (+672)</v>
-      </c>
-      <c r="B103" s="1" t="str">
-        <v>NF</v>
-      </c>
-      <c r="C103" s="1" t="str">
-        <v>+672</v>
-      </c>
-    </row>
-    <row r="104" ht="23" customHeight="1">
-      <c r="A104" s="1" t="str">
-        <v>Islandia (+354)</v>
-      </c>
-      <c r="B104" s="1" t="str">
-        <v>IS</v>
-      </c>
-      <c r="C104" s="1" t="str">
-        <v>+354</v>
-      </c>
-    </row>
-    <row r="105" ht="23" customHeight="1">
-      <c r="A105" s="1" t="str">
-        <v>Islas Aland (+358)</v>
-      </c>
-      <c r="B105" s="1" t="str">
-        <v>AX</v>
-      </c>
-      <c r="C105" s="1" t="str">
-        <v>+358</v>
-      </c>
-    </row>
-    <row r="106" ht="23" customHeight="1">
-      <c r="A106" s="1" t="str">
-        <v>Islas Caimán (+1)</v>
-      </c>
-      <c r="B106" s="1" t="str">
-        <v>KY</v>
-      </c>
-      <c r="C106" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="107" ht="23" customHeight="1">
-      <c r="A107" s="1" t="str">
-        <v>Islas Cocos (+61)</v>
-      </c>
-      <c r="B107" s="1" t="str">
-        <v>CC</v>
-      </c>
-      <c r="C107" s="1" t="str">
-        <v>+61</v>
-      </c>
-    </row>
-    <row r="108" ht="23" customHeight="1">
-      <c r="A108" s="1" t="str">
-        <v>Islas Cook (+682)</v>
-      </c>
-      <c r="B108" s="1" t="str">
-        <v>CK</v>
-      </c>
-      <c r="C108" s="1" t="str">
-        <v>+682</v>
-      </c>
-    </row>
-    <row r="109" ht="23" customHeight="1">
-      <c r="A109" s="1" t="str">
-        <v>Islas Feroe (+298)</v>
-      </c>
-      <c r="B109" s="1" t="str">
-        <v>FO</v>
-      </c>
-      <c r="C109" s="1" t="str">
-        <v>+298</v>
-      </c>
-    </row>
-    <row r="110" ht="23" customHeight="1">
-      <c r="A110" s="1" t="str">
-        <v>Islas Malvinas (+500)</v>
-      </c>
-      <c r="B110" s="1" t="str">
-        <v>FK</v>
-      </c>
-      <c r="C110" s="1" t="str">
-        <v>+500</v>
-      </c>
-    </row>
-    <row r="111" ht="23" customHeight="1">
-      <c r="A111" s="1" t="str">
-        <v>Islas Marianas del Norte (+1)</v>
-      </c>
-      <c r="B111" s="1" t="str">
-        <v>MP</v>
-      </c>
-      <c r="C111" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="112" ht="23" customHeight="1">
-      <c r="A112" s="1" t="str">
-        <v>Islas Marshall (+692)</v>
-      </c>
-      <c r="B112" s="1" t="str">
-        <v>MH</v>
-      </c>
-      <c r="C112" s="1" t="str">
-        <v>+692</v>
-      </c>
-    </row>
-    <row r="113" ht="23" customHeight="1">
-      <c r="A113" s="1" t="str">
-        <v>Islas Salomón (+677)</v>
-      </c>
-      <c r="B113" s="1" t="str">
-        <v>SB</v>
-      </c>
-      <c r="C113" s="1" t="str">
-        <v>+677</v>
-      </c>
-    </row>
-    <row r="114" ht="23" customHeight="1">
-      <c r="A114" s="1" t="str">
-        <v>Islas Turcas y Caicos (+1)</v>
-      </c>
-      <c r="B114" s="1" t="str">
-        <v>TC</v>
-      </c>
-      <c r="C114" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="115" ht="23" customHeight="1">
-      <c r="A115" s="1" t="str">
-        <v>Islas Vírgenes Británicas (+1)</v>
-      </c>
-      <c r="B115" s="1" t="str">
-        <v>VG</v>
-      </c>
-      <c r="C115" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="116" ht="23" customHeight="1">
-      <c r="A116" s="1" t="str">
-        <v>Islas Vírgenes de EE. UU. (+1)</v>
-      </c>
-      <c r="B116" s="1" t="str">
-        <v>VI</v>
-      </c>
-      <c r="C116" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="117" ht="23" customHeight="1">
-      <c r="A117" s="1" t="str">
-        <v>Israel (+972)</v>
-      </c>
-      <c r="B117" s="1" t="str">
-        <v>IL</v>
-      </c>
-      <c r="C117" s="1" t="str">
-        <v>+972</v>
-      </c>
-    </row>
-    <row r="118" ht="23" customHeight="1">
-      <c r="A118" s="1" t="str">
-        <v>Italia (+39)</v>
-      </c>
-      <c r="B118" s="1" t="str">
-        <v>IT</v>
-      </c>
-      <c r="C118" s="1" t="str">
-        <v>+39</v>
-      </c>
-    </row>
-    <row r="119" ht="23" customHeight="1">
-      <c r="A119" s="1" t="str">
-        <v>Jamaica (+1)</v>
-      </c>
-      <c r="B119" s="1" t="str">
-        <v>JM</v>
-      </c>
-      <c r="C119" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="120" ht="23" customHeight="1">
-      <c r="A120" s="1" t="str">
-        <v>Japón (+81)</v>
-      </c>
-      <c r="B120" s="1" t="str">
-        <v>JP</v>
-      </c>
-      <c r="C120" s="1" t="str">
-        <v>+81</v>
-      </c>
-    </row>
-    <row r="121" ht="23" customHeight="1">
-      <c r="A121" s="1" t="str">
-        <v>Jersey (+44)</v>
-      </c>
-      <c r="B121" s="1" t="str">
-        <v>JE</v>
-      </c>
-      <c r="C121" s="1" t="str">
-        <v>+44</v>
-      </c>
-    </row>
-    <row r="122" ht="23" customHeight="1">
-      <c r="A122" s="1" t="str">
-        <v>Jordania (+962)</v>
-      </c>
-      <c r="B122" s="1" t="str">
-        <v>JO</v>
-      </c>
-      <c r="C122" s="1" t="str">
-        <v>+962</v>
-      </c>
-    </row>
-    <row r="123" ht="23" customHeight="1">
-      <c r="A123" s="1" t="str">
-        <v>Kazajistán (+7)</v>
-      </c>
-      <c r="B123" s="1" t="str">
-        <v>KZ</v>
-      </c>
-      <c r="C123" s="1" t="str">
-        <v>+7</v>
-      </c>
-    </row>
-    <row r="124" ht="23" customHeight="1">
-      <c r="A124" s="1" t="str">
-        <v>Kenia (+254)</v>
-      </c>
-      <c r="B124" s="1" t="str">
-        <v>KE</v>
-      </c>
-      <c r="C124" s="1" t="str">
-        <v>+254</v>
-      </c>
-    </row>
-    <row r="125" ht="23" customHeight="1">
-      <c r="A125" s="1" t="str">
-        <v>Kirguistán (+996)</v>
-      </c>
-      <c r="B125" s="1" t="str">
-        <v>KG</v>
-      </c>
-      <c r="C125" s="1" t="str">
-        <v>+996</v>
-      </c>
-    </row>
-    <row r="126" ht="23" customHeight="1">
-      <c r="A126" s="1" t="str">
-        <v>Kiribati (+686)</v>
-      </c>
-      <c r="B126" s="1" t="str">
-        <v>KI</v>
-      </c>
-      <c r="C126" s="1" t="str">
-        <v>+686</v>
-      </c>
-    </row>
-    <row r="127" ht="23" customHeight="1">
-      <c r="A127" s="1" t="str">
-        <v>Kosovo (+383)</v>
-      </c>
-      <c r="B127" s="1" t="str">
-        <v>XK</v>
-      </c>
-      <c r="C127" s="1" t="str">
-        <v>+383</v>
-      </c>
-    </row>
-    <row r="128" ht="23" customHeight="1">
-      <c r="A128" s="1" t="str">
-        <v>Kuwait (+965)</v>
-      </c>
-      <c r="B128" s="1" t="str">
-        <v>KW</v>
-      </c>
-      <c r="C128" s="1" t="str">
-        <v>+965</v>
-      </c>
-    </row>
-    <row r="129" ht="23" customHeight="1">
-      <c r="A129" s="1" t="str">
-        <v>Laos (+856)</v>
-      </c>
-      <c r="B129" s="1" t="str">
-        <v>LA</v>
-      </c>
-      <c r="C129" s="1" t="str">
-        <v>+856</v>
-      </c>
-    </row>
-    <row r="130" ht="23" customHeight="1">
-      <c r="A130" s="1" t="str">
-        <v>Lesoto (+266)</v>
-      </c>
-      <c r="B130" s="1" t="str">
-        <v>LS</v>
-      </c>
-      <c r="C130" s="1" t="str">
-        <v>+266</v>
-      </c>
-    </row>
-    <row r="131" ht="23" customHeight="1">
-      <c r="A131" s="1" t="str">
-        <v>Letonia (+371)</v>
-      </c>
-      <c r="B131" s="1" t="str">
-        <v>LV</v>
-      </c>
-      <c r="C131" s="1" t="str">
-        <v>+371</v>
-      </c>
-    </row>
-    <row r="132" ht="23" customHeight="1">
-      <c r="A132" s="1" t="str">
-        <v>Líbano (+961)</v>
-      </c>
-      <c r="B132" s="1" t="str">
-        <v>LB</v>
-      </c>
-      <c r="C132" s="1" t="str">
-        <v>+961</v>
-      </c>
-    </row>
-    <row r="133" ht="23" customHeight="1">
-      <c r="A133" s="1" t="str">
-        <v>Liberia (+231)</v>
-      </c>
-      <c r="B133" s="1" t="str">
-        <v>LR</v>
-      </c>
-      <c r="C133" s="1" t="str">
-        <v>+231</v>
-      </c>
-    </row>
-    <row r="134" ht="23" customHeight="1">
-      <c r="A134" s="1" t="str">
-        <v>Libia (+218)</v>
-      </c>
-      <c r="B134" s="1" t="str">
-        <v>LY</v>
-      </c>
-      <c r="C134" s="1" t="str">
-        <v>+218</v>
-      </c>
-    </row>
-    <row r="135" ht="23" customHeight="1">
-      <c r="A135" s="1" t="str">
-        <v>Liechtenstein (+423)</v>
-      </c>
-      <c r="B135" s="1" t="str">
-        <v>LI</v>
-      </c>
-      <c r="C135" s="1" t="str">
-        <v>+423</v>
-      </c>
-    </row>
-    <row r="136" ht="23" customHeight="1">
-      <c r="A136" s="1" t="str">
-        <v>Lituania (+370)</v>
-      </c>
-      <c r="B136" s="1" t="str">
-        <v>LT</v>
-      </c>
-      <c r="C136" s="1" t="str">
-        <v>+370</v>
-      </c>
-    </row>
-    <row r="137" ht="23" customHeight="1">
-      <c r="A137" s="1" t="str">
-        <v>Luxemburgo (+352)</v>
-      </c>
-      <c r="B137" s="1" t="str">
-        <v>LU</v>
-      </c>
-      <c r="C137" s="1" t="str">
-        <v>+352</v>
-      </c>
-    </row>
-    <row r="138" ht="23" customHeight="1">
-      <c r="A138" s="1" t="str">
-        <v>Macedonia del Norte (+389)</v>
-      </c>
-      <c r="B138" s="1" t="str">
-        <v>MK</v>
-      </c>
-      <c r="C138" s="1" t="str">
-        <v>+389</v>
-      </c>
-    </row>
-    <row r="139" ht="23" customHeight="1">
-      <c r="A139" s="1" t="str">
-        <v>Madagascar (+261)</v>
-      </c>
-      <c r="B139" s="1" t="str">
-        <v>MG</v>
-      </c>
-      <c r="C139" s="1" t="str">
-        <v>+261</v>
-      </c>
-    </row>
-    <row r="140" ht="23" customHeight="1">
-      <c r="A140" s="1" t="str">
-        <v>Malasia (+60)</v>
-      </c>
-      <c r="B140" s="1" t="str">
-        <v>MY</v>
-      </c>
-      <c r="C140" s="1" t="str">
-        <v>+60</v>
-      </c>
-    </row>
-    <row r="141" ht="23" customHeight="1">
-      <c r="A141" s="1" t="str">
-        <v>Malaui (+265)</v>
-      </c>
-      <c r="B141" s="1" t="str">
-        <v>MW</v>
-      </c>
-      <c r="C141" s="1" t="str">
-        <v>+265</v>
-      </c>
-    </row>
-    <row r="142" ht="23" customHeight="1">
-      <c r="A142" s="1" t="str">
-        <v>Maldivas (+960)</v>
-      </c>
-      <c r="B142" s="1" t="str">
-        <v>MV</v>
-      </c>
-      <c r="C142" s="1" t="str">
-        <v>+960</v>
-      </c>
-    </row>
-    <row r="143" ht="23" customHeight="1">
-      <c r="A143" s="1" t="str">
-        <v>Mali (+223)</v>
-      </c>
-      <c r="B143" s="1" t="str">
-        <v>ML</v>
-      </c>
-      <c r="C143" s="1" t="str">
-        <v>+223</v>
-      </c>
-    </row>
-    <row r="144" ht="23" customHeight="1">
-      <c r="A144" s="1" t="str">
-        <v>Malta (+356)</v>
-      </c>
-      <c r="B144" s="1" t="str">
-        <v>MT</v>
-      </c>
-      <c r="C144" s="1" t="str">
-        <v>+356</v>
-      </c>
-    </row>
-    <row r="145" ht="23" customHeight="1">
-      <c r="A145" s="1" t="str">
-        <v>Marruecos (+212)</v>
-      </c>
-      <c r="B145" s="1" t="str">
-        <v>MA</v>
-      </c>
-      <c r="C145" s="1" t="str">
-        <v>+212</v>
-      </c>
-    </row>
-    <row r="146" ht="23" customHeight="1">
-      <c r="A146" s="1" t="str">
-        <v>Martinica (+596)</v>
-      </c>
-      <c r="B146" s="1" t="str">
-        <v>MQ</v>
-      </c>
-      <c r="C146" s="1" t="str">
-        <v>+596</v>
-      </c>
-    </row>
-    <row r="147" ht="23" customHeight="1">
-      <c r="A147" s="1" t="str">
-        <v>Mauricio (+230)</v>
-      </c>
-      <c r="B147" s="1" t="str">
-        <v>MU</v>
-      </c>
-      <c r="C147" s="1" t="str">
-        <v>+230</v>
-      </c>
-    </row>
-    <row r="148" ht="23" customHeight="1">
-      <c r="A148" s="1" t="str">
-        <v>Mauritania (+222)</v>
-      </c>
-      <c r="B148" s="1" t="str">
-        <v>MR</v>
-      </c>
-      <c r="C148" s="1" t="str">
-        <v>+222</v>
-      </c>
-    </row>
-    <row r="149" ht="23" customHeight="1">
-      <c r="A149" s="1" t="str">
-        <v>Mayotte (+262)</v>
-      </c>
-      <c r="B149" s="1" t="str">
-        <v>YT</v>
-      </c>
-      <c r="C149" s="1" t="str">
-        <v>+262</v>
-      </c>
-    </row>
-    <row r="150" ht="23" customHeight="1">
-      <c r="A150" s="1" t="str">
-        <v>México (+52)</v>
-      </c>
-      <c r="B150" s="1" t="str">
-        <v>MX</v>
-      </c>
-      <c r="C150" s="1" t="str">
-        <v>+52</v>
-      </c>
-    </row>
-    <row r="151" ht="23" customHeight="1">
-      <c r="A151" s="1" t="str">
-        <v>Micronesia (+691)</v>
-      </c>
-      <c r="B151" s="1" t="str">
-        <v>FM</v>
-      </c>
-      <c r="C151" s="1" t="str">
-        <v>+691</v>
-      </c>
-    </row>
-    <row r="152" ht="23" customHeight="1">
-      <c r="A152" s="1" t="str">
-        <v>Moldavia (+373)</v>
-      </c>
-      <c r="B152" s="1" t="str">
-        <v>MD</v>
-      </c>
-      <c r="C152" s="1" t="str">
-        <v>+373</v>
-      </c>
-    </row>
-    <row r="153" ht="23" customHeight="1">
-      <c r="A153" s="1" t="str">
-        <v>Mónaco (+377)</v>
-      </c>
-      <c r="B153" s="1" t="str">
-        <v>MC</v>
-      </c>
-      <c r="C153" s="1" t="str">
-        <v>+377</v>
-      </c>
-    </row>
-    <row r="154" ht="23" customHeight="1">
-      <c r="A154" s="1" t="str">
-        <v>Mongolia (+976)</v>
-      </c>
-      <c r="B154" s="1" t="str">
-        <v>MN</v>
-      </c>
-      <c r="C154" s="1" t="str">
-        <v>+976</v>
-      </c>
-    </row>
-    <row r="155" ht="23" customHeight="1">
-      <c r="A155" s="1" t="str">
-        <v>Montenegro (+382)</v>
-      </c>
-      <c r="B155" s="1" t="str">
-        <v>ME</v>
-      </c>
-      <c r="C155" s="1" t="str">
-        <v>+382</v>
-      </c>
-    </row>
-    <row r="156" ht="23" customHeight="1">
-      <c r="A156" s="1" t="str">
-        <v>Montserrat (+1)</v>
-      </c>
-      <c r="B156" s="1" t="str">
-        <v>MS</v>
-      </c>
-      <c r="C156" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="157" ht="23" customHeight="1">
-      <c r="A157" s="1" t="str">
-        <v>Mozambique (+258)</v>
-      </c>
-      <c r="B157" s="1" t="str">
-        <v>MZ</v>
-      </c>
-      <c r="C157" s="1" t="str">
-        <v>+258</v>
-      </c>
-    </row>
-    <row r="158" ht="23" customHeight="1">
-      <c r="A158" s="1" t="str">
-        <v>Myanmar (Birmania) (+95)</v>
-      </c>
-      <c r="B158" s="1" t="str">
-        <v>MM</v>
-      </c>
-      <c r="C158" s="1" t="str">
-        <v>+95</v>
-      </c>
-    </row>
-    <row r="159" ht="23" customHeight="1">
-      <c r="A159" s="1" t="str">
-        <v>Namibia (+264)</v>
-      </c>
-      <c r="B159" s="1" t="str">
-        <v>NA</v>
-      </c>
-      <c r="C159" s="1" t="str">
-        <v>+264</v>
-      </c>
-    </row>
-    <row r="160" ht="23" customHeight="1">
-      <c r="A160" s="1" t="str">
-        <v>Nauru (+674)</v>
-      </c>
-      <c r="B160" s="1" t="str">
-        <v>NR</v>
-      </c>
-      <c r="C160" s="1" t="str">
-        <v>+674</v>
-      </c>
-    </row>
-    <row r="161" ht="23" customHeight="1">
-      <c r="A161" s="1" t="str">
-        <v>Nepal (+977)</v>
-      </c>
-      <c r="B161" s="1" t="str">
-        <v>NP</v>
-      </c>
-      <c r="C161" s="1" t="str">
-        <v>+977</v>
-      </c>
-    </row>
-    <row r="162" ht="23" customHeight="1">
-      <c r="A162" s="1" t="str">
-        <v>Nicaragua (+505)</v>
-      </c>
-      <c r="B162" s="1" t="str">
-        <v>NI</v>
-      </c>
-      <c r="C162" s="1" t="str">
-        <v>+505</v>
-      </c>
-    </row>
-    <row r="163" ht="23" customHeight="1">
-      <c r="A163" s="1" t="str">
-        <v>Níger (+227)</v>
-      </c>
-      <c r="B163" s="1" t="str">
-        <v>NE</v>
-      </c>
-      <c r="C163" s="1" t="str">
-        <v>+227</v>
-      </c>
-    </row>
-    <row r="164" ht="23" customHeight="1">
-      <c r="A164" s="1" t="str">
-        <v>Nigeria (+234)</v>
-      </c>
-      <c r="B164" s="1" t="str">
-        <v>NG</v>
-      </c>
-      <c r="C164" s="1" t="str">
-        <v>+234</v>
-      </c>
-    </row>
-    <row r="165" ht="23" customHeight="1">
-      <c r="A165" s="1" t="str">
-        <v>Niue (+683)</v>
-      </c>
-      <c r="B165" s="1" t="str">
-        <v>NU</v>
-      </c>
-      <c r="C165" s="1" t="str">
-        <v>+683</v>
-      </c>
-    </row>
-    <row r="166" ht="23" customHeight="1">
-      <c r="A166" s="1" t="str">
-        <v>Noruega (+47)</v>
-      </c>
-      <c r="B166" s="1" t="str">
-        <v>NO</v>
-      </c>
-      <c r="C166" s="1" t="str">
-        <v>+47</v>
-      </c>
-    </row>
-    <row r="167" ht="23" customHeight="1">
-      <c r="A167" s="1" t="str">
-        <v>Nueva Caledonia (+687)</v>
-      </c>
-      <c r="B167" s="1" t="str">
-        <v>NC</v>
-      </c>
-      <c r="C167" s="1" t="str">
-        <v>+687</v>
-      </c>
-    </row>
-    <row r="168" ht="23" customHeight="1">
-      <c r="A168" s="1" t="str">
-        <v>Nueva Zelanda (+64)</v>
-      </c>
-      <c r="B168" s="1" t="str">
-        <v>NZ</v>
-      </c>
-      <c r="C168" s="1" t="str">
-        <v>+64</v>
-      </c>
-    </row>
-    <row r="169" ht="23" customHeight="1">
-      <c r="A169" s="1" t="str">
-        <v>Omán (+968)</v>
-      </c>
-      <c r="B169" s="1" t="str">
-        <v>OM</v>
-      </c>
-      <c r="C169" s="1" t="str">
-        <v>+968</v>
-      </c>
-    </row>
-    <row r="170" ht="23" customHeight="1">
-      <c r="A170" s="1" t="str">
-        <v>Países Bajos (+31)</v>
-      </c>
-      <c r="B170" s="1" t="str">
-        <v>NL</v>
-      </c>
-      <c r="C170" s="1" t="str">
-        <v>+31</v>
-      </c>
-    </row>
-    <row r="171" ht="23" customHeight="1">
-      <c r="A171" s="1" t="str">
-        <v>Pakistán (+92)</v>
-      </c>
-      <c r="B171" s="1" t="str">
-        <v>PK</v>
-      </c>
-      <c r="C171" s="1" t="str">
-        <v>+92</v>
-      </c>
-    </row>
-    <row r="172" ht="23" customHeight="1">
-      <c r="A172" s="1" t="str">
-        <v>Palaos (+680)</v>
-      </c>
-      <c r="B172" s="1" t="str">
-        <v>PW</v>
-      </c>
-      <c r="C172" s="1" t="str">
-        <v>+680</v>
-      </c>
-    </row>
-    <row r="173" ht="23" customHeight="1">
-      <c r="A173" s="1" t="str">
-        <v>Panamá (+507)</v>
-      </c>
-      <c r="B173" s="1" t="str">
-        <v>PA</v>
-      </c>
-      <c r="C173" s="1" t="str">
-        <v>+507</v>
-      </c>
-    </row>
-    <row r="174" ht="23" customHeight="1">
-      <c r="A174" s="1" t="str">
-        <v>Papúa Nueva Guinea (+675)</v>
-      </c>
-      <c r="B174" s="1" t="str">
-        <v>PG</v>
-      </c>
-      <c r="C174" s="1" t="str">
-        <v>+675</v>
-      </c>
-    </row>
-    <row r="175" ht="23" customHeight="1">
-      <c r="A175" s="1" t="str">
-        <v>Paraguay (+595)</v>
-      </c>
-      <c r="B175" s="1" t="str">
-        <v>PY</v>
-      </c>
-      <c r="C175" s="1" t="str">
-        <v>+595</v>
-      </c>
-    </row>
-    <row r="176" ht="23" customHeight="1">
-      <c r="A176" s="1" t="str">
-        <v>Perú (+51)</v>
-      </c>
-      <c r="B176" s="1" t="str">
-        <v>PE</v>
-      </c>
-      <c r="C176" s="1" t="str">
-        <v>+51</v>
-      </c>
-    </row>
-    <row r="177" ht="23" customHeight="1">
-      <c r="A177" s="1" t="str">
-        <v>Polinesia Francesa (+689)</v>
-      </c>
-      <c r="B177" s="1" t="str">
-        <v>PF</v>
-      </c>
-      <c r="C177" s="1" t="str">
-        <v>+689</v>
-      </c>
-    </row>
-    <row r="178" ht="23" customHeight="1">
-      <c r="A178" s="1" t="str">
-        <v>Polonia (+48)</v>
-      </c>
-      <c r="B178" s="1" t="str">
-        <v>PL</v>
-      </c>
-      <c r="C178" s="1" t="str">
-        <v>+48</v>
-      </c>
-    </row>
-    <row r="179" ht="23" customHeight="1">
-      <c r="A179" s="1" t="str">
-        <v>Portugal (+351)</v>
-      </c>
-      <c r="B179" s="1" t="str">
-        <v>PT</v>
-      </c>
-      <c r="C179" s="1" t="str">
-        <v>+351</v>
-      </c>
-    </row>
-    <row r="180" ht="23" customHeight="1">
-      <c r="A180" s="1" t="str">
-        <v>Puerto Rico (+1)</v>
-      </c>
-      <c r="B180" s="1" t="str">
-        <v>PR</v>
-      </c>
-      <c r="C180" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="181" ht="23" customHeight="1">
-      <c r="A181" s="1" t="str">
-        <v>RAE de Hong Kong (China) (+852)</v>
-      </c>
-      <c r="B181" s="1" t="str">
-        <v>HK</v>
-      </c>
-      <c r="C181" s="1" t="str">
-        <v>+852</v>
-      </c>
-    </row>
-    <row r="182" ht="23" customHeight="1">
-      <c r="A182" s="1" t="str">
-        <v>RAE de Macao (China) (+853)</v>
-      </c>
-      <c r="B182" s="1" t="str">
-        <v>MO</v>
-      </c>
-      <c r="C182" s="1" t="str">
-        <v>+853</v>
-      </c>
-    </row>
-    <row r="183" ht="23" customHeight="1">
-      <c r="A183" s="1" t="str">
-        <v>Reino Unido (+44)</v>
-      </c>
-      <c r="B183" s="1" t="str">
-        <v>GB</v>
-      </c>
-      <c r="C183" s="1" t="str">
-        <v>+44</v>
-      </c>
-    </row>
-    <row r="184" ht="23" customHeight="1">
-      <c r="A184" s="1" t="str">
-        <v>República Centroafricana (+236)</v>
-      </c>
-      <c r="B184" s="1" t="str">
-        <v>CF</v>
-      </c>
-      <c r="C184" s="1" t="str">
-        <v>+236</v>
-      </c>
-    </row>
-    <row r="185" ht="23" customHeight="1">
-      <c r="A185" s="1" t="str">
-        <v>República Democrática del Congo (+243)</v>
-      </c>
-      <c r="B185" s="1" t="str">
-        <v>CD</v>
-      </c>
-      <c r="C185" s="1" t="str">
-        <v>+243</v>
-      </c>
-    </row>
-    <row r="186" ht="23" customHeight="1">
-      <c r="A186" s="1" t="str">
-        <v>República Dominicana (+1)</v>
-      </c>
-      <c r="B186" s="1" t="str">
-        <v>DO</v>
-      </c>
-      <c r="C186" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="187" ht="23" customHeight="1">
-      <c r="A187" s="1" t="str">
-        <v>Reunión (+262)</v>
-      </c>
-      <c r="B187" s="1" t="str">
-        <v>RE</v>
-      </c>
-      <c r="C187" s="1" t="str">
-        <v>+262</v>
-      </c>
-    </row>
-    <row r="188" ht="23" customHeight="1">
-      <c r="A188" s="1" t="str">
-        <v>Ruanda (+250)</v>
-      </c>
-      <c r="B188" s="1" t="str">
-        <v>RW</v>
-      </c>
-      <c r="C188" s="1" t="str">
-        <v>+250</v>
-      </c>
-    </row>
-    <row r="189" ht="23" customHeight="1">
-      <c r="A189" s="1" t="str">
-        <v>Rumanía (+40)</v>
-      </c>
-      <c r="B189" s="1" t="str">
-        <v>RO</v>
-      </c>
-      <c r="C189" s="1" t="str">
-        <v>+40</v>
-      </c>
-    </row>
-    <row r="190" ht="23" customHeight="1">
-      <c r="A190" s="1" t="str">
-        <v>Rusia (+7)</v>
-      </c>
-      <c r="B190" s="1" t="str">
-        <v>RU</v>
-      </c>
-      <c r="C190" s="1" t="str">
-        <v>+7</v>
-      </c>
-    </row>
-    <row r="191" ht="23" customHeight="1">
-      <c r="A191" s="1" t="str">
-        <v>Sáhara Occidental (+212)</v>
-      </c>
-      <c r="B191" s="1" t="str">
-        <v>EH</v>
-      </c>
-      <c r="C191" s="1" t="str">
-        <v>+212</v>
-      </c>
-    </row>
-    <row r="192" ht="23" customHeight="1">
-      <c r="A192" s="1" t="str">
-        <v>Samoa (+685)</v>
-      </c>
-      <c r="B192" s="1" t="str">
-        <v>WS</v>
-      </c>
-      <c r="C192" s="1" t="str">
-        <v>+685</v>
-      </c>
-    </row>
-    <row r="193" ht="23" customHeight="1">
-      <c r="A193" s="1" t="str">
-        <v>Samoa Americana (+1)</v>
-      </c>
-      <c r="B193" s="1" t="str">
-        <v>AS</v>
-      </c>
-      <c r="C193" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="194" ht="23" customHeight="1">
-      <c r="A194" s="1" t="str">
-        <v>San Bartolomé (+590)</v>
-      </c>
-      <c r="B194" s="1" t="str">
-        <v>BL</v>
-      </c>
-      <c r="C194" s="1" t="str">
-        <v>+590</v>
-      </c>
-    </row>
-    <row r="195" ht="23" customHeight="1">
-      <c r="A195" s="1" t="str">
-        <v>San Cristóbal y Nieves (+1)</v>
-      </c>
-      <c r="B195" s="1" t="str">
-        <v>KN</v>
-      </c>
-      <c r="C195" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="196" ht="23" customHeight="1">
-      <c r="A196" s="1" t="str">
-        <v>San Marino (+378)</v>
-      </c>
-      <c r="B196" s="1" t="str">
-        <v>SM</v>
-      </c>
-      <c r="C196" s="1" t="str">
-        <v>+378</v>
-      </c>
-    </row>
-    <row r="197" ht="23" customHeight="1">
-      <c r="A197" s="1" t="str">
-        <v>San Martín (+590)</v>
-      </c>
-      <c r="B197" s="1" t="str">
-        <v>MF</v>
-      </c>
-      <c r="C197" s="1" t="str">
-        <v>+590</v>
-      </c>
-    </row>
-    <row r="198" ht="23" customHeight="1">
-      <c r="A198" s="1" t="str">
-        <v>San Pedro y Miquelón (+508)</v>
-      </c>
-      <c r="B198" s="1" t="str">
-        <v>PM</v>
-      </c>
-      <c r="C198" s="1" t="str">
-        <v>+508</v>
-      </c>
-    </row>
-    <row r="199" ht="23" customHeight="1">
-      <c r="A199" s="1" t="str">
-        <v>San Vicente y las Granadinas (+1)</v>
-      </c>
-      <c r="B199" s="1" t="str">
-        <v>VC</v>
-      </c>
-      <c r="C199" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="200" ht="23" customHeight="1">
-      <c r="A200" s="1" t="str">
-        <v>Santa Elena (+290)</v>
-      </c>
-      <c r="B200" s="1" t="str">
-        <v>SH</v>
-      </c>
-      <c r="C200" s="1" t="str">
-        <v>+290</v>
-      </c>
-    </row>
-    <row r="201" ht="23" customHeight="1">
-      <c r="A201" s="1" t="str">
-        <v>Santa Lucía (+1)</v>
-      </c>
-      <c r="B201" s="1" t="str">
-        <v>LC</v>
-      </c>
-      <c r="C201" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="202" ht="23" customHeight="1">
-      <c r="A202" s="1" t="str">
-        <v>Santo Tomé y Príncipe (+239)</v>
-      </c>
-      <c r="B202" s="1" t="str">
-        <v>ST</v>
-      </c>
-      <c r="C202" s="1" t="str">
-        <v>+239</v>
-      </c>
-    </row>
-    <row r="203" ht="23" customHeight="1">
-      <c r="A203" s="1" t="str">
-        <v>Senegal (+221)</v>
-      </c>
-      <c r="B203" s="1" t="str">
-        <v>SN</v>
-      </c>
-      <c r="C203" s="1" t="str">
-        <v>+221</v>
-      </c>
-    </row>
-    <row r="204" ht="23" customHeight="1">
-      <c r="A204" s="1" t="str">
-        <v>Serbia (+381)</v>
-      </c>
-      <c r="B204" s="1" t="str">
-        <v>RS</v>
-      </c>
-      <c r="C204" s="1" t="str">
-        <v>+381</v>
-      </c>
-    </row>
-    <row r="205" ht="23" customHeight="1">
-      <c r="A205" s="1" t="str">
-        <v>Seychelles (+248)</v>
-      </c>
-      <c r="B205" s="1" t="str">
-        <v>SC</v>
-      </c>
-      <c r="C205" s="1" t="str">
-        <v>+248</v>
-      </c>
-    </row>
-    <row r="206" ht="23" customHeight="1">
-      <c r="A206" s="1" t="str">
-        <v>Sierra Leona (+232)</v>
-      </c>
-      <c r="B206" s="1" t="str">
-        <v>SL</v>
-      </c>
-      <c r="C206" s="1" t="str">
-        <v>+232</v>
-      </c>
-    </row>
-    <row r="207" ht="23" customHeight="1">
-      <c r="A207" s="1" t="str">
-        <v>Singapur (+65)</v>
-      </c>
-      <c r="B207" s="1" t="str">
-        <v>SG</v>
-      </c>
-      <c r="C207" s="1" t="str">
-        <v>+65</v>
-      </c>
-    </row>
-    <row r="208" ht="23" customHeight="1">
-      <c r="A208" s="1" t="str">
-        <v>Sint Maarten (+1)</v>
-      </c>
-      <c r="B208" s="1" t="str">
-        <v>SX</v>
-      </c>
-      <c r="C208" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="209" ht="23" customHeight="1">
-      <c r="A209" s="1" t="str">
-        <v>Siria (+963)</v>
-      </c>
-      <c r="B209" s="1" t="str">
-        <v>SY</v>
-      </c>
-      <c r="C209" s="1" t="str">
-        <v>+963</v>
-      </c>
-    </row>
-    <row r="210" ht="23" customHeight="1">
-      <c r="A210" s="1" t="str">
-        <v>Somalia (+252)</v>
-      </c>
-      <c r="B210" s="1" t="str">
-        <v>SO</v>
-      </c>
-      <c r="C210" s="1" t="str">
-        <v>+252</v>
-      </c>
-    </row>
-    <row r="211" ht="23" customHeight="1">
-      <c r="A211" s="1" t="str">
-        <v>Sri Lanka (+94)</v>
-      </c>
-      <c r="B211" s="1" t="str">
-        <v>LK</v>
-      </c>
-      <c r="C211" s="1" t="str">
-        <v>+94</v>
-      </c>
-    </row>
-    <row r="212" ht="23" customHeight="1">
-      <c r="A212" s="1" t="str">
-        <v>Sudáfrica (+27)</v>
-      </c>
-      <c r="B212" s="1" t="str">
-        <v>ZA</v>
-      </c>
-      <c r="C212" s="1" t="str">
-        <v>+27</v>
-      </c>
-    </row>
-    <row r="213" ht="23" customHeight="1">
-      <c r="A213" s="1" t="str">
-        <v>Sudán (+249)</v>
-      </c>
-      <c r="B213" s="1" t="str">
-        <v>SD</v>
-      </c>
-      <c r="C213" s="1" t="str">
-        <v>+249</v>
-      </c>
-    </row>
-    <row r="214" ht="23" customHeight="1">
-      <c r="A214" s="1" t="str">
-        <v>Sudán del Sur (+211)</v>
-      </c>
-      <c r="B214" s="1" t="str">
-        <v>SS</v>
-      </c>
-      <c r="C214" s="1" t="str">
-        <v>+211</v>
-      </c>
-    </row>
-    <row r="215" ht="23" customHeight="1">
-      <c r="A215" s="1" t="str">
-        <v>Suecia (+46)</v>
-      </c>
-      <c r="B215" s="1" t="str">
-        <v>SE</v>
-      </c>
-      <c r="C215" s="1" t="str">
-        <v>+46</v>
-      </c>
-    </row>
-    <row r="216" ht="23" customHeight="1">
-      <c r="A216" s="1" t="str">
-        <v>Suiza (+41)</v>
-      </c>
-      <c r="B216" s="1" t="str">
-        <v>CH</v>
-      </c>
-      <c r="C216" s="1" t="str">
-        <v>+41</v>
-      </c>
-    </row>
-    <row r="217" ht="23" customHeight="1">
-      <c r="A217" s="1" t="str">
-        <v>Surinam (+597)</v>
-      </c>
-      <c r="B217" s="1" t="str">
-        <v>SR</v>
-      </c>
-      <c r="C217" s="1" t="str">
-        <v>+597</v>
-      </c>
-    </row>
-    <row r="218" ht="23" customHeight="1">
-      <c r="A218" s="1" t="str">
-        <v>Svalbard y Jan Mayen (+47)</v>
-      </c>
-      <c r="B218" s="1" t="str">
-        <v>SJ</v>
-      </c>
-      <c r="C218" s="1" t="str">
-        <v>+47</v>
-      </c>
-    </row>
-    <row r="219" ht="23" customHeight="1">
-      <c r="A219" s="1" t="str">
-        <v>Tailandia (+66)</v>
-      </c>
-      <c r="B219" s="1" t="str">
-        <v>TH</v>
-      </c>
-      <c r="C219" s="1" t="str">
-        <v>+66</v>
-      </c>
-    </row>
-    <row r="220" ht="23" customHeight="1">
-      <c r="A220" s="1" t="str">
-        <v>Taiwán (+886)</v>
-      </c>
-      <c r="B220" s="1" t="str">
-        <v>TW</v>
-      </c>
-      <c r="C220" s="1" t="str">
-        <v>+886</v>
-      </c>
-    </row>
-    <row r="221" ht="23" customHeight="1">
-      <c r="A221" s="1" t="str">
-        <v>Tanzania (+255)</v>
-      </c>
-      <c r="B221" s="1" t="str">
-        <v>TZ</v>
-      </c>
-      <c r="C221" s="1" t="str">
-        <v>+255</v>
-      </c>
-    </row>
-    <row r="222" ht="23" customHeight="1">
-      <c r="A222" s="1" t="str">
-        <v>Tayikistán (+992)</v>
-      </c>
-      <c r="B222" s="1" t="str">
-        <v>TJ</v>
-      </c>
-      <c r="C222" s="1" t="str">
-        <v>+992</v>
-      </c>
-    </row>
-    <row r="223" ht="23" customHeight="1">
-      <c r="A223" s="1" t="str">
-        <v>Territorio Británico del Océano Índico (+246)</v>
-      </c>
-      <c r="B223" s="1" t="str">
-        <v>IO</v>
-      </c>
-      <c r="C223" s="1" t="str">
-        <v>+246</v>
-      </c>
-    </row>
-    <row r="224" ht="23" customHeight="1">
-      <c r="A224" s="1" t="str">
-        <v>Territorios Palestinos (+970)</v>
-      </c>
-      <c r="B224" s="1" t="str">
-        <v>PS</v>
-      </c>
-      <c r="C224" s="1" t="str">
-        <v>+970</v>
-      </c>
-    </row>
-    <row r="225" ht="23" customHeight="1">
-      <c r="A225" s="1" t="str">
-        <v>Timor-Leste (+670)</v>
-      </c>
-      <c r="B225" s="1" t="str">
-        <v>TL</v>
-      </c>
-      <c r="C225" s="1" t="str">
-        <v>+670</v>
-      </c>
-    </row>
-    <row r="226" ht="23" customHeight="1">
-      <c r="A226" s="1" t="str">
-        <v>Togo (+228)</v>
-      </c>
-      <c r="B226" s="1" t="str">
-        <v>TG</v>
-      </c>
-      <c r="C226" s="1" t="str">
-        <v>+228</v>
-      </c>
-    </row>
-    <row r="227" ht="23" customHeight="1">
-      <c r="A227" s="1" t="str">
-        <v>Tokelau (+690)</v>
-      </c>
-      <c r="B227" s="1" t="str">
-        <v>TK</v>
-      </c>
-      <c r="C227" s="1" t="str">
-        <v>+690</v>
-      </c>
-    </row>
-    <row r="228" ht="23" customHeight="1">
-      <c r="A228" s="1" t="str">
-        <v>Tonga (+676)</v>
-      </c>
-      <c r="B228" s="1" t="str">
-        <v>TO</v>
-      </c>
-      <c r="C228" s="1" t="str">
-        <v>+676</v>
-      </c>
-    </row>
-    <row r="229" ht="23" customHeight="1">
-      <c r="A229" s="1" t="str">
-        <v>Trinidad y Tobago (+1)</v>
-      </c>
-      <c r="B229" s="1" t="str">
-        <v>TT</v>
-      </c>
-      <c r="C229" s="1" t="str">
-        <v>+1</v>
-      </c>
-    </row>
-    <row r="230" ht="23" customHeight="1">
-      <c r="A230" s="1" t="str">
-        <v>Tristán de Acuña (+290)</v>
-      </c>
-      <c r="B230" s="1" t="str">
-        <v>TA</v>
-      </c>
-      <c r="C230" s="1" t="str">
-        <v>+290</v>
-      </c>
-    </row>
-    <row r="231" ht="23" customHeight="1">
-      <c r="A231" s="1" t="str">
-        <v>Túnez (+216)</v>
-      </c>
-      <c r="B231" s="1" t="str">
-        <v>TN</v>
-      </c>
-      <c r="C231" s="1" t="str">
-        <v>+216</v>
-      </c>
-    </row>
-    <row r="232" ht="23" customHeight="1">
-      <c r="A232" s="1" t="str">
-        <v>Turkmenistán (+993)</v>
-      </c>
-      <c r="B232" s="1" t="str">
-        <v>TM</v>
-      </c>
-      <c r="C232" s="1" t="str">
-        <v>+993</v>
-      </c>
-    </row>
-    <row r="233" ht="23" customHeight="1">
-      <c r="A233" s="1" t="str">
-        <v>Turquía (+90)</v>
-      </c>
-      <c r="B233" s="1" t="str">
-        <v>TR</v>
-      </c>
-      <c r="C233" s="1" t="str">
-        <v>+90</v>
-      </c>
-    </row>
-    <row r="234" ht="23" customHeight="1">
-      <c r="A234" s="1" t="str">
-        <v>Tuvalu (+688)</v>
-      </c>
-      <c r="B234" s="1" t="str">
-        <v>TV</v>
-      </c>
-      <c r="C234" s="1" t="str">
-        <v>+688</v>
-      </c>
-    </row>
-    <row r="235" ht="23" customHeight="1">
-      <c r="A235" s="1" t="str">
-        <v>Ucrania (+380)</v>
-      </c>
-      <c r="B235" s="1" t="str">
-        <v>UA</v>
-      </c>
-      <c r="C235" s="1" t="str">
-        <v>+380</v>
-      </c>
-    </row>
-    <row r="236" ht="23" customHeight="1">
-      <c r="A236" s="1" t="str">
-        <v>Uganda (+256)</v>
-      </c>
-      <c r="B236" s="1" t="str">
-        <v>UG</v>
-      </c>
-      <c r="C236" s="1" t="str">
-        <v>+256</v>
-      </c>
-    </row>
-    <row r="237" ht="23" customHeight="1">
-      <c r="A237" s="1" t="str">
-        <v>Uruguay (+598)</v>
-      </c>
-      <c r="B237" s="1" t="str">
-        <v>UY</v>
-      </c>
-      <c r="C237" s="1" t="str">
-        <v>+598</v>
-      </c>
-    </row>
-    <row r="238" ht="23" customHeight="1">
-      <c r="A238" s="1" t="str">
-        <v>Uzbekistán (+998)</v>
-      </c>
-      <c r="B238" s="1" t="str">
-        <v>UZ</v>
-      </c>
-      <c r="C238" s="1" t="str">
-        <v>+998</v>
-      </c>
-    </row>
-    <row r="239" ht="23" customHeight="1">
-      <c r="A239" s="1" t="str">
-        <v>Vanuatu (+678)</v>
-      </c>
-      <c r="B239" s="1" t="str">
-        <v>VU</v>
-      </c>
-      <c r="C239" s="1" t="str">
-        <v>+678</v>
-      </c>
-    </row>
-    <row r="240" ht="23" customHeight="1">
-      <c r="A240" s="1" t="str">
-        <v>Venezuela (+58)</v>
-      </c>
-      <c r="B240" s="1" t="str">
-        <v>VE</v>
-      </c>
-      <c r="C240" s="1" t="str">
         <v>+58</v>
-      </c>
-    </row>
-    <row r="241" ht="23" customHeight="1">
-      <c r="A241" s="1" t="str">
-        <v>Vietnam (+84)</v>
-      </c>
-      <c r="B241" s="1" t="str">
-        <v>VN</v>
-      </c>
-      <c r="C241" s="1" t="str">
-        <v>+84</v>
-      </c>
-    </row>
-    <row r="242" ht="23" customHeight="1">
-      <c r="A242" s="1" t="str">
-        <v>Wallis y Futuna (+681)</v>
-      </c>
-      <c r="B242" s="1" t="str">
-        <v>WF</v>
-      </c>
-      <c r="C242" s="1" t="str">
-        <v>+681</v>
-      </c>
-    </row>
-    <row r="243" ht="23" customHeight="1">
-      <c r="A243" s="1" t="str">
-        <v>Yemen (+967)</v>
-      </c>
-      <c r="B243" s="1" t="str">
-        <v>YE</v>
-      </c>
-      <c r="C243" s="1" t="str">
-        <v>+967</v>
-      </c>
-    </row>
-    <row r="244" ht="23" customHeight="1">
-      <c r="A244" s="1" t="str">
-        <v>Yibuti (+253)</v>
-      </c>
-      <c r="B244" s="1" t="str">
-        <v>DJ</v>
-      </c>
-      <c r="C244" s="1" t="str">
-        <v>+253</v>
-      </c>
-    </row>
-    <row r="245" ht="23" customHeight="1">
-      <c r="A245" s="1" t="str">
-        <v>Zambia (+260)</v>
-      </c>
-      <c r="B245" s="1" t="str">
-        <v>ZM</v>
-      </c>
-      <c r="C245" s="1" t="str">
-        <v>+260</v>
-      </c>
-    </row>
-    <row r="246" ht="23" customHeight="1">
-      <c r="A246" s="1" t="str">
-        <v>Zimbabue (+263)</v>
-      </c>
-      <c r="B246" s="1" t="str">
-        <v>ZW</v>
-      </c>
-      <c r="C246" s="1" t="str">
-        <v>+263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Keep confirmed couples together and seat guests by category
</commit_message>
<xml_diff>
--- a/public/templates/plantilla-invitados.xlsx
+++ b/public/templates/plantilla-invitados.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Invitados" sheetId="1" r:id="R8ec6eedff6db497f"/>
-    <sheet name="Países" sheetId="2" r:id="Rc3469867abcc486d" state="hidden"/>
+    <sheet name="Invitados" sheetId="1" r:id="Rc13b9a1b57f243bf"/>
+    <sheet name="Países" sheetId="2" r:id="R1458ffc1df224aee" state="hidden"/>
   </sheets>
   <definedNames>
     <definedName name="PaisesTelefonicos">'Países'!$A$2:$A$22</definedName>
@@ -250,14 +250,14 @@
   <dxfs count="2">
     <dxf>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFFCE8E4"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFFCE8E4"/>
         </patternFill>
       </fill>
@@ -6620,17 +6620,17 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation type="list" sqref="D5" showErrorMessage="1" errorStyle="stop" errorTitle="Elige una opción" error="Selecciona una opción del desplegable." showInputMessage="1" promptTitle="Empieza aquí" prompt="Elige el país de la mayoría de tus invitados.">
+    <dataValidation type="list" errorStyle="stop" showInputMessage="1" showErrorMessage="1" errorTitle="Elige una opción" error="Selecciona una opción del desplegable." promptTitle="Empieza aquí" prompt="Elige el país de la mayoría de tus invitados." sqref="D5">
       <formula1>PaisesTelefonicos</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="D11:D510" showErrorMessage="1" errorStyle="stop" errorTitle="Elige una opción" error="Selecciona una opción del desplegable.">
+    <dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="Elige una opción" error="Selecciona una opción del desplegable." sqref="D11:D510">
       <formula1>PaisesTelefonicos</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="F11:F510" showErrorMessage="1" errorStyle="stop" errorTitle="Elige una opción" error="Selecciona una opción del desplegable.">
+    <dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="Elige una opción" error="Selecciona una opción del desplegable." sqref="F11:F510">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="G11:G510" showErrorMessage="1" errorStyle="stop" errorTitle="Elige una opción" error="Selecciona una opción del desplegable.">
-      <formula1>"Familia del novio,Familia de la novia,Amigos del novio,Amigos de la novia,Amigos,Compañeros de trabajo,Otros"</formula1>
+    <dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="Elige una opción" error="Selecciona una opción del desplegable." sqref="G11:G510">
+      <formula1>"Familia del novio,Familia de la novia,Amigos del novio,Amigos de la novia,Amigos,Compañeros de trabajo,Compañeros de trabajo del novio,Compañeros de trabajo de la novia,Otros"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>